<commit_message>
attach-document.vbs: take the company code into account (optional CC / Company Code column)
The company code is entered on the XK03 start screen so SAP validates the vendor
in that company code; the done list and log include it. Example workbook updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BfnV7zbTBY9KHu4eQyf6JQ
</commit_message>
<xml_diff>
--- a/sap-attach/examples/attachment-only example.xlsx
+++ b/sap-attach/examples/attachment-only example.xlsx
@@ -418,7 +418,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -430,7 +430,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vendor Name</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -445,10 +445,12 @@
           <t>0002020008</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>1265</v>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:\Users\290158\Downloads\Scripts\RE_ Suspensiones hasta nuevo aviso.msg</t>
+          <t>RE_ Suspensiones hasta nuevo aviso.msg</t>
         </is>
       </c>
     </row>

</xml_diff>